<commit_message>
Updates to first sheets
</commit_message>
<xml_diff>
--- a/output/IMG_9688.xlsx
+++ b/output/IMG_9688.xlsx
@@ -902,7 +902,7 @@
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>ドライ・マッシュ ポテト(ふ・ポ風味)造粒品</t>
+          <t>ドライ・マッシュ ポテト(ふ・ぱい風味)造粒品</t>
         </is>
       </c>
       <c r="E6" s="12" t="n"/>
@@ -1123,7 +1123,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>GE0006280        999 購入
+          <t>GB0006280        999 購入
 Shayco 『80-ポテューズ2ポテ』</t>
         </is>
       </c>
@@ -1162,7 +1162,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>GE0005150        999 購入
+          <t>GB0005150        999 購入
 IATA INSTANT COFFEE FR-2132(微粉り)</t>
         </is>
       </c>
@@ -1201,7 +1201,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>GE0004220        999 購入
+          <t>GB0004220        999 購入
 鎌塚レシダー</t>
         </is>
       </c>
@@ -1240,7 +1240,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>GE0003040        999 購入
+          <t>GB0003040        999 購入
 ステラス×200(大茂植食)</t>
         </is>
       </c>
@@ -1279,7 +1279,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>GE0002070        999 購入
+          <t>GB0002070        999 購入
 フッジ K-EM.</t>
         </is>
       </c>
@@ -1318,7 +1318,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>GE0003110        999 購入
+          <t>GB0003110        999 購入
 ボエムZ 1-3</t>
         </is>
       </c>
@@ -1357,8 +1357,8 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>GE0006810        999 購入
-ハダーー『ミナーズ SSH-181</t>
+          <t>GB0006810        999 購入
+ハダーー『 ミナチュー SSH-181</t>
         </is>
       </c>
       <c r="B18" s="12" t="n"/>
@@ -1396,8 +1396,8 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t>GE0004800        999 購入
-コーヒー ダターブレーデー YM-5309</t>
+          <t>GB0004800        999 購入
+コーヒー ダダーブレーダー YM-5309</t>
         </is>
       </c>
       <c r="B19" s="12" t="n"/>

</xml_diff>

<commit_message>
Sheets type 3 and part of 4 template implementatino
</commit_message>
<xml_diff>
--- a/output/IMG_9688.xlsx
+++ b/output/IMG_9688.xlsx
@@ -742,7 +742,7 @@
       <c r="C2" s="6" t="n"/>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>0000056481</t>
+          <t>0000056481 1</t>
         </is>
       </c>
       <c r="E2" s="5" t="n"/>
@@ -757,7 +757,7 @@
       <c r="J2" s="6" t="n"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>2018/12/06</t>
+          <t>2018/12/05</t>
         </is>
       </c>
       <c r="L2" s="5" t="n"/>
@@ -810,7 +810,7 @@
       <c r="C4" s="10" t="n"/>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>S00000200 製造1課 倉庫</t>
+          <t>S00000200 製造１課 倉庫</t>
         </is>
       </c>
       <c r="E4" s="9" t="n"/>
@@ -902,7 +902,7 @@
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>ドライ・マッシュ ポテト(ふ・ポ風味)造粒品</t>
+          <t>クレイジーマックスプロテイン（カフェオレ風味）造粒品</t>
         </is>
       </c>
       <c r="E6" s="12" t="n"/>
@@ -966,7 +966,7 @@
       <c r="Q7" s="13" t="n"/>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>S00000200 製造1課 倉庫</t>
+          <t>S00000200 製造１課 倉庫</t>
         </is>
       </c>
       <c r="S7" s="12" t="n"/>
@@ -984,11 +984,7 @@
       </c>
       <c r="B8" s="12" t="n"/>
       <c r="C8" s="13" t="n"/>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>0000056481</t>
-        </is>
-      </c>
+      <c r="D8" s="12" t="n"/>
       <c r="E8" s="12" t="n"/>
       <c r="F8" s="12" t="n"/>
       <c r="G8" s="12" t="n"/>
@@ -1123,8 +1119,8 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>GE0006280        999 購入
-Shayco 『80-ポテューズ2ポテ』</t>
+          <t>GE0006280
+Wheyco W80-パフォーマンスアカデミー</t>
         </is>
       </c>
       <c r="B12" s="26" t="n"/>
@@ -1139,17 +1135,22 @@
       <c r="K12" s="27" t="n"/>
       <c r="L12" s="28" t="inlineStr">
         <is>
-          <t>89.8383</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M12" s="27" t="n"/>
       <c r="N12" s="28" t="inlineStr">
         <is>
-          <t>360.00 kg</t>
+          <t>89.8383</t>
         </is>
       </c>
       <c r="O12" s="27" t="n"/>
-      <c r="P12" s="28" t="n"/>
+      <c r="P12" s="28" t="inlineStr">
+        <is>
+          <t>360.00
+kg</t>
+        </is>
+      </c>
       <c r="Q12" s="27" t="n"/>
       <c r="R12" s="28" t="n"/>
       <c r="S12" s="26" t="n"/>
@@ -1162,8 +1163,8 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>GE0005150        999 購入
-IATA INSTANT COFFEE FR-2132(微粉り)</t>
+          <t>GE0005150
+TATA INSTANT COFFEE FR-2132（深煎り）</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
@@ -1178,17 +1179,22 @@
       <c r="K13" s="13" t="n"/>
       <c r="L13" s="11" t="inlineStr">
         <is>
-          <t>5.9893</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>24.00 kg</t>
+          <t>5.9893</t>
         </is>
       </c>
       <c r="O13" s="13" t="n"/>
-      <c r="P13" s="11" t="n"/>
+      <c r="P13" s="11" t="inlineStr">
+        <is>
+          <t>24.00
+kg</t>
+        </is>
+      </c>
       <c r="Q13" s="13" t="n"/>
       <c r="R13" s="11" t="n"/>
       <c r="S13" s="12" t="n"/>
@@ -1201,8 +1207,8 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>GE0004220        999 購入
-鎌塚レシピダー</t>
+          <t>GE0004220
+練乳パウダー</t>
         </is>
       </c>
       <c r="B14" s="12" t="n"/>
@@ -1217,17 +1223,22 @@
       <c r="K14" s="13" t="n"/>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>2.2959</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="11" t="inlineStr">
         <is>
-          <t>9.20 kg</t>
+          <t>2.2959</t>
         </is>
       </c>
       <c r="O14" s="13" t="n"/>
-      <c r="P14" s="11" t="n"/>
+      <c r="P14" s="11" t="inlineStr">
+        <is>
+          <t>9.20
+kg</t>
+        </is>
+      </c>
       <c r="Q14" s="13" t="n"/>
       <c r="R14" s="11" t="n"/>
       <c r="S14" s="12" t="n"/>
@@ -1240,8 +1251,8 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>GE0003040        999 購入
-ステラス×200(大宮機食)</t>
+          <t>GE0003040
+ステラロース200（大宮糧食）</t>
         </is>
       </c>
       <c r="B15" s="12" t="n"/>
@@ -1256,17 +1267,22 @@
       <c r="K15" s="13" t="n"/>
       <c r="L15" s="11" t="inlineStr">
         <is>
-          <t>0.2795</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M15" s="13" t="n"/>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>1.12 kg</t>
+          <t>0.2795</t>
         </is>
       </c>
       <c r="O15" s="13" t="n"/>
-      <c r="P15" s="11" t="n"/>
+      <c r="P15" s="11" t="inlineStr">
+        <is>
+          <t>1.12
+kg</t>
+        </is>
+      </c>
       <c r="Q15" s="13" t="n"/>
       <c r="R15" s="11" t="n"/>
       <c r="S15" s="12" t="n"/>
@@ -1279,8 +1295,8 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>GE0002070        999 購入
-フッジ K-EM.</t>
+          <t>GE0002070
+ソレック K-EML</t>
         </is>
       </c>
       <c r="B16" s="12" t="n"/>
@@ -1295,17 +1311,22 @@
       <c r="K16" s="13" t="n"/>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>0.2995</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>1.20 kg</t>
+          <t>0.2995</t>
         </is>
       </c>
       <c r="O16" s="13" t="n"/>
-      <c r="P16" s="11" t="n"/>
+      <c r="P16" s="11" t="inlineStr">
+        <is>
+          <t>1.20
+kg</t>
+        </is>
+      </c>
       <c r="Q16" s="13" t="n"/>
       <c r="R16" s="11" t="n"/>
       <c r="S16" s="12" t="n"/>
@@ -1318,8 +1339,8 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>GE0003110        999 購入
-ボエムZ 1-3</t>
+          <t>GE0003110
+ポエムＺＬ－３</t>
         </is>
       </c>
       <c r="B17" s="12" t="n"/>
@@ -1334,17 +1355,22 @@
       <c r="K17" s="13" t="n"/>
       <c r="L17" s="11" t="inlineStr">
         <is>
-          <t>0.4991</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M17" s="13" t="n"/>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>2.00 kg</t>
+          <t>0.4991</t>
         </is>
       </c>
       <c r="O17" s="13" t="n"/>
-      <c r="P17" s="11" t="n"/>
+      <c r="P17" s="11" t="inlineStr">
+        <is>
+          <t>2.00
+kg</t>
+        </is>
+      </c>
       <c r="Q17" s="13" t="n"/>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="12" t="n"/>
@@ -1357,8 +1383,8 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>GE0006810        999 購入
-ハダーロー ミナーズ SSH-181</t>
+          <t>GE0006810
+バクダードミルクコーヒー SSH-181</t>
         </is>
       </c>
       <c r="B18" s="12" t="n"/>
@@ -1373,17 +1399,22 @@
       <c r="K18" s="13" t="n"/>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>0.4991</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M18" s="13" t="n"/>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>2.00 kg</t>
+          <t>0.4991</t>
         </is>
       </c>
       <c r="O18" s="13" t="n"/>
-      <c r="P18" s="11" t="n"/>
+      <c r="P18" s="11" t="inlineStr">
+        <is>
+          <t>2.00
+kg</t>
+        </is>
+      </c>
       <c r="Q18" s="13" t="n"/>
       <c r="R18" s="11" t="n"/>
       <c r="S18" s="12" t="n"/>
@@ -1396,8 +1427,8 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t>GE0004800        999 購入
-コーヒー ダターフレーバー YM-5309</t>
+          <t>GE0004800
+コーヒーパウダーフレーバー YM-5309</t>
         </is>
       </c>
       <c r="B19" s="12" t="n"/>
@@ -1412,17 +1443,22 @@
       <c r="K19" s="13" t="n"/>
       <c r="L19" s="11" t="inlineStr">
         <is>
-          <t>0.2995</t>
+          <t>999 購入</t>
         </is>
       </c>
       <c r="M19" s="13" t="n"/>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>1.20 kg</t>
+          <t>0.2995</t>
         </is>
       </c>
       <c r="O19" s="13" t="n"/>
-      <c r="P19" s="11" t="n"/>
+      <c r="P19" s="11" t="inlineStr">
+        <is>
+          <t>1.20
+kg</t>
+        </is>
+      </c>
       <c r="Q19" s="13" t="n"/>
       <c r="R19" s="11" t="n"/>
       <c r="S19" s="12" t="n"/>

</xml_diff>

<commit_message>
Merge fixes D:, and almost done with second to last sheet style
</commit_message>
<xml_diff>
--- a/output/IMG_9688.xlsx
+++ b/output/IMG_9688.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="製造指図書" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,16 +27,20 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="12"/>
     </font>
     <font>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="00000000"/>
       <sz val="22"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -742,7 +746,7 @@
       <c r="C2" s="6" t="n"/>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>0000056481 1</t>
+          <t>0000056481　1</t>
         </is>
       </c>
       <c r="E2" s="5" t="n"/>
@@ -810,7 +814,7 @@
       <c r="C4" s="10" t="n"/>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>S00000200 製造１課 倉庫</t>
+          <t>S00000200 製造１課　倉庫</t>
         </is>
       </c>
       <c r="E4" s="9" t="n"/>
@@ -944,7 +948,7 @@
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>20 仕込</t>
+          <t>20　仕込</t>
         </is>
       </c>
       <c r="E7" s="12" t="n"/>
@@ -966,7 +970,7 @@
       <c r="Q7" s="13" t="n"/>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>S00000200 製造１課 倉庫</t>
+          <t>S00000200 製造１課　倉庫</t>
         </is>
       </c>
       <c r="S7" s="12" t="n"/>
@@ -1119,7 +1123,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>GE0006280
+          <t>GE0006280        999 購入
 Wheyco W80-パフォーマンスアカデミー</t>
         </is>
       </c>
@@ -1135,22 +1139,18 @@
       <c r="K12" s="27" t="n"/>
       <c r="L12" s="28" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>89.8383</t>
         </is>
       </c>
       <c r="M12" s="27" t="n"/>
       <c r="N12" s="28" t="inlineStr">
         <is>
-          <t>89.8383</t>
-        </is>
-      </c>
-      <c r="O12" s="27" t="n"/>
-      <c r="P12" s="28" t="inlineStr">
-        <is>
           <t>360.00
 kg</t>
         </is>
       </c>
+      <c r="O12" s="27" t="n"/>
+      <c r="P12" s="28" t="n"/>
       <c r="Q12" s="27" t="n"/>
       <c r="R12" s="28" t="n"/>
       <c r="S12" s="26" t="n"/>
@@ -1163,7 +1163,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>GE0005150
+          <t>GE0005150        999 購入
 TATA INSTANT COFFEE FR-2132（深煎り）</t>
         </is>
       </c>
@@ -1179,22 +1179,18 @@
       <c r="K13" s="13" t="n"/>
       <c r="L13" s="11" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>5.9893</t>
         </is>
       </c>
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>5.9893</t>
-        </is>
-      </c>
-      <c r="O13" s="13" t="n"/>
-      <c r="P13" s="11" t="inlineStr">
-        <is>
           <t>24.00
 kg</t>
         </is>
       </c>
+      <c r="O13" s="13" t="n"/>
+      <c r="P13" s="11" t="n"/>
       <c r="Q13" s="13" t="n"/>
       <c r="R13" s="11" t="n"/>
       <c r="S13" s="12" t="n"/>
@@ -1207,7 +1203,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>GE0004220
+          <t>GE0004220        999 購入
 練乳パウダー</t>
         </is>
       </c>
@@ -1223,22 +1219,18 @@
       <c r="K14" s="13" t="n"/>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>2.2959</t>
         </is>
       </c>
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="11" t="inlineStr">
         <is>
-          <t>2.2959</t>
-        </is>
-      </c>
-      <c r="O14" s="13" t="n"/>
-      <c r="P14" s="11" t="inlineStr">
-        <is>
           <t>9.20
 kg</t>
         </is>
       </c>
+      <c r="O14" s="13" t="n"/>
+      <c r="P14" s="11" t="n"/>
       <c r="Q14" s="13" t="n"/>
       <c r="R14" s="11" t="n"/>
       <c r="S14" s="12" t="n"/>
@@ -1251,7 +1243,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>GE0003040
+          <t>GE0003040        999 購入
 ステラロース200（大宮糧食）</t>
         </is>
       </c>
@@ -1267,22 +1259,18 @@
       <c r="K15" s="13" t="n"/>
       <c r="L15" s="11" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>0.2795</t>
         </is>
       </c>
       <c r="M15" s="13" t="n"/>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>0.2795</t>
-        </is>
-      </c>
-      <c r="O15" s="13" t="n"/>
-      <c r="P15" s="11" t="inlineStr">
-        <is>
           <t>1.12
 kg</t>
         </is>
       </c>
+      <c r="O15" s="13" t="n"/>
+      <c r="P15" s="11" t="n"/>
       <c r="Q15" s="13" t="n"/>
       <c r="R15" s="11" t="n"/>
       <c r="S15" s="12" t="n"/>
@@ -1295,7 +1283,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>GE0002070
+          <t>GE0002070        999 購入
 ソレック K-EML</t>
         </is>
       </c>
@@ -1311,22 +1299,18 @@
       <c r="K16" s="13" t="n"/>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>0.2995</t>
         </is>
       </c>
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>0.2995</t>
-        </is>
-      </c>
-      <c r="O16" s="13" t="n"/>
-      <c r="P16" s="11" t="inlineStr">
-        <is>
           <t>1.20
 kg</t>
         </is>
       </c>
+      <c r="O16" s="13" t="n"/>
+      <c r="P16" s="11" t="n"/>
       <c r="Q16" s="13" t="n"/>
       <c r="R16" s="11" t="n"/>
       <c r="S16" s="12" t="n"/>
@@ -1339,7 +1323,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>GE0003110
+          <t>GE0003110        999 購入
 ポエムＺＬ－３</t>
         </is>
       </c>
@@ -1355,22 +1339,18 @@
       <c r="K17" s="13" t="n"/>
       <c r="L17" s="11" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>0.4991</t>
         </is>
       </c>
       <c r="M17" s="13" t="n"/>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>0.4991</t>
-        </is>
-      </c>
-      <c r="O17" s="13" t="n"/>
-      <c r="P17" s="11" t="inlineStr">
-        <is>
           <t>2.00
 kg</t>
         </is>
       </c>
+      <c r="O17" s="13" t="n"/>
+      <c r="P17" s="11" t="n"/>
       <c r="Q17" s="13" t="n"/>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="12" t="n"/>
@@ -1383,7 +1363,7 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>GE0006810
+          <t>GE0006810        999 購入
 バクダードミルクコーヒー SSH-181</t>
         </is>
       </c>
@@ -1399,22 +1379,18 @@
       <c r="K18" s="13" t="n"/>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>0.4991</t>
         </is>
       </c>
       <c r="M18" s="13" t="n"/>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>0.4991</t>
-        </is>
-      </c>
-      <c r="O18" s="13" t="n"/>
-      <c r="P18" s="11" t="inlineStr">
-        <is>
           <t>2.00
 kg</t>
         </is>
       </c>
+      <c r="O18" s="13" t="n"/>
+      <c r="P18" s="11" t="n"/>
       <c r="Q18" s="13" t="n"/>
       <c r="R18" s="11" t="n"/>
       <c r="S18" s="12" t="n"/>
@@ -1427,7 +1403,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t>GE0004800
+          <t>GE0004800        999 購入
 コーヒーパウダーフレーバー YM-5309</t>
         </is>
       </c>
@@ -1443,22 +1419,18 @@
       <c r="K19" s="13" t="n"/>
       <c r="L19" s="11" t="inlineStr">
         <is>
-          <t>999 購入</t>
+          <t>0.2995</t>
         </is>
       </c>
       <c r="M19" s="13" t="n"/>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>0.2995</t>
-        </is>
-      </c>
-      <c r="O19" s="13" t="n"/>
-      <c r="P19" s="11" t="inlineStr">
-        <is>
           <t>1.20
 kg</t>
         </is>
       </c>
+      <c r="O19" s="13" t="n"/>
+      <c r="P19" s="11" t="n"/>
       <c r="Q19" s="13" t="n"/>
       <c r="R19" s="11" t="n"/>
       <c r="S19" s="12" t="n"/>

</xml_diff>

<commit_message>
templates except for 9693
</commit_message>
<xml_diff>
--- a/output/IMG_9688.xlsx
+++ b/output/IMG_9688.xlsx
@@ -1130,7 +1130,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>GE0006280        999 購入
+          <t>GE0006280
 Wheyco W80-パフォーマンスアカデミー</t>
         </is>
       </c>
@@ -1146,7 +1146,8 @@
       <c r="K12" s="28" t="n"/>
       <c r="L12" s="29" t="inlineStr">
         <is>
-          <t>89.8383</t>
+          <t>999 購入
+89.8383</t>
         </is>
       </c>
       <c r="M12" s="28" t="n"/>
@@ -1170,7 +1171,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>GE0005150        999 購入
+          <t>GE0005150
 TATA INSTANT COFFEE FR-2132（深煎り）</t>
         </is>
       </c>
@@ -1186,7 +1187,8 @@
       <c r="K13" s="14" t="n"/>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>5.9893</t>
+          <t>999 購入
+5.9893</t>
         </is>
       </c>
       <c r="M13" s="14" t="n"/>
@@ -1210,7 +1212,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>GE0004220        999 購入
+          <t>GE0004220
 練乳パウダー</t>
         </is>
       </c>
@@ -1226,7 +1228,8 @@
       <c r="K14" s="14" t="n"/>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>2.2959</t>
+          <t>999 購入
+2.2959</t>
         </is>
       </c>
       <c r="M14" s="14" t="n"/>
@@ -1250,8 +1253,8 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="30" t="inlineStr">
         <is>
-          <t>GE0003040        999 購入
-ステラロース200（大宮糧食）</t>
+          <t>GE0003040
+スタラース200（大宮糧食）</t>
         </is>
       </c>
       <c r="B15" s="13" t="n"/>
@@ -1266,7 +1269,8 @@
       <c r="K15" s="14" t="n"/>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>0.2795</t>
+          <t>999 購入
+0.2795</t>
         </is>
       </c>
       <c r="M15" s="14" t="n"/>
@@ -1290,7 +1294,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>GE0002070        999 購入
+          <t>GE0002070
 アレック K-EML</t>
         </is>
       </c>
@@ -1306,7 +1310,8 @@
       <c r="K16" s="14" t="n"/>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>0.2995</t>
+          <t>999 購入
+0.2995</t>
         </is>
       </c>
       <c r="M16" s="14" t="n"/>
@@ -1330,8 +1335,8 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>GE0003110        999 購入
-ポエムZ L－3</t>
+          <t>GE0003110
+ポエムＺＬ－３</t>
         </is>
       </c>
       <c r="B17" s="13" t="n"/>
@@ -1346,7 +1351,8 @@
       <c r="K17" s="14" t="n"/>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>0.4991</t>
+          <t>999 購入
+0.4991</t>
         </is>
       </c>
       <c r="M17" s="14" t="n"/>
@@ -1370,8 +1376,8 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>GE0006810        999 購入
-バクダードミルクコーヒー SSH-181</t>
+          <t>GE0006810
+パウダートミルクコーヒー SSH-181</t>
         </is>
       </c>
       <c r="B18" s="13" t="n"/>
@@ -1386,7 +1392,8 @@
       <c r="K18" s="14" t="n"/>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>0.4991</t>
+          <t>999 購入
+0.4991</t>
         </is>
       </c>
       <c r="M18" s="14" t="n"/>
@@ -1410,7 +1417,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>GE0004800        999 購入
+          <t>GE0004800
 コーヒーパウダーフレーバー YM-5309</t>
         </is>
       </c>
@@ -1426,7 +1433,8 @@
       <c r="K19" s="14" t="n"/>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>0.2995</t>
+          <t>999 購入
+0.2995</t>
         </is>
       </c>
       <c r="M19" s="14" t="n"/>

</xml_diff>